<commit_message>
Update shop UI and save detail
</commit_message>
<xml_diff>
--- a/Game/Data/Locale/Locale.xlsx
+++ b/Game/Data/Locale/Locale.xlsx
@@ -2566,6 +2566,17 @@
         <x:v>完成</x:v>
       </x:c>
     </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>price</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>Price</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Fix bugs about domain and update editor preview
</commit_message>
<xml_diff>
--- a/Game/Data/Locale/Locale.xlsx
+++ b/Game/Data/Locale/Locale.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fengmingliu/Dev/Ludork/Game/Data/Locale/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E770E48-2E83-0743-A834-FE41AB3D8771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B179700D-C7BD-904B-BD70-2052D1D6F179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -1451,12 +1451,6 @@
     <t>S_DOMAIN_DESC</t>
   </si>
   <si>
-    <t>After each player move, the enemy deals one-round damage while the player is within its {value}-cell Manhattan range.</t>
-  </si>
-  <si>
-    <t>玩家每次移动后，若处于敌人的{value}格曼哈顿领域范围内，敌人造成一次单回合伤害。</t>
-  </si>
-  <si>
     <t>S_FLANK</t>
   </si>
   <si>
@@ -1887,6 +1881,12 @@
   </si>
   <si>
     <t>点击此头像可打开菜单。</t>
+  </si>
+  <si>
+    <t>玩家每次移动后，若处于敌人的{value}格范围内，敌人造成一次单回合伤害。</t>
+  </si>
+  <si>
+    <t>After each player move, the enemy deals one-round damage while the player is within its {value}-cell range.</t>
   </si>
 </sst>
 </file>
@@ -1903,26 +1903,36 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1953,7 +1963,7 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3062,143 +3072,143 @@
       <c r="A17" t="s">
         <v>471</v>
       </c>
-      <c r="B17" t="s">
-        <v>472</v>
-      </c>
-      <c r="C17" t="s">
-        <v>473</v>
+      <c r="B17" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>616</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>472</v>
+      </c>
+      <c r="B18" t="s">
+        <v>473</v>
+      </c>
+      <c r="C18" t="s">
         <v>474</v>
-      </c>
-      <c r="B18" t="s">
-        <v>475</v>
-      </c>
-      <c r="C18" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>475</v>
+      </c>
+      <c r="B19" t="s">
+        <v>476</v>
+      </c>
+      <c r="C19" t="s">
         <v>477</v>
-      </c>
-      <c r="B19" t="s">
-        <v>478</v>
-      </c>
-      <c r="C19" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>478</v>
+      </c>
+      <c r="B20" t="s">
+        <v>479</v>
+      </c>
+      <c r="C20" t="s">
         <v>480</v>
-      </c>
-      <c r="B20" t="s">
-        <v>481</v>
-      </c>
-      <c r="C20" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
+        <v>481</v>
+      </c>
+      <c r="B21" t="s">
+        <v>482</v>
+      </c>
+      <c r="C21" t="s">
         <v>483</v>
-      </c>
-      <c r="B21" t="s">
-        <v>484</v>
-      </c>
-      <c r="C21" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>486</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>487</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>489</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>490</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>490</v>
+      </c>
+      <c r="B24" t="s">
+        <v>491</v>
+      </c>
+      <c r="C24" t="s">
         <v>492</v>
-      </c>
-      <c r="B24" t="s">
-        <v>493</v>
-      </c>
-      <c r="C24" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>493</v>
+      </c>
+      <c r="B25" t="s">
+        <v>494</v>
+      </c>
+      <c r="C25" t="s">
         <v>495</v>
-      </c>
-      <c r="B25" t="s">
-        <v>496</v>
-      </c>
-      <c r="C25" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="B26" t="s">
+        <v>497</v>
+      </c>
+      <c r="C26" t="s">
         <v>498</v>
-      </c>
-      <c r="B26" t="s">
-        <v>499</v>
-      </c>
-      <c r="C26" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="B27" t="s">
+        <v>500</v>
+      </c>
+      <c r="C27" t="s">
         <v>501</v>
-      </c>
-      <c r="B27" t="s">
-        <v>502</v>
-      </c>
-      <c r="C27" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
+        <v>502</v>
+      </c>
+      <c r="B28" t="s">
+        <v>503</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>504</v>
-      </c>
-      <c r="B28" t="s">
-        <v>505</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
+        <v>505</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>507</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>508</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>509</v>
       </c>
     </row>
   </sheetData>
@@ -3228,24 +3238,24 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B2" t="s">
+        <v>509</v>
+      </c>
+      <c r="C2" t="s">
         <v>510</v>
-      </c>
-      <c r="B2" t="s">
-        <v>511</v>
-      </c>
-      <c r="C2" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>511</v>
+      </c>
+      <c r="B3" t="s">
+        <v>512</v>
+      </c>
+      <c r="C3" t="s">
         <v>513</v>
-      </c>
-      <c r="B3" t="s">
-        <v>514</v>
-      </c>
-      <c r="C3" t="s">
-        <v>515</v>
       </c>
     </row>
   </sheetData>
@@ -3276,35 +3286,35 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>516</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>517</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>519</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>520</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>522</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>524</v>
       </c>
     </row>
   </sheetData>
@@ -3333,134 +3343,134 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>525</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>526</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>528</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>529</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>531</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>532</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>534</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>535</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>537</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>538</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>540</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>541</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>543</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>545</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>546</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>547</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>549</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>550</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>551</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>552</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>553</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>554</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>555</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>556</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>557</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>558</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>559</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="122.75" customHeight="1"/>
@@ -3505,211 +3515,211 @@
     </row>
     <row r="2" spans="1:3" ht="64">
       <c r="A2" s="8" t="s">
+        <v>559</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>561</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>562</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>563</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="48">
       <c r="A3" s="8" t="s">
+        <v>562</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>563</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>564</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>565</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>566</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="64">
       <c r="A4" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>566</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>567</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>568</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>569</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="96">
       <c r="A5" s="8" t="s">
+        <v>568</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>569</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>570</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>571</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="64">
       <c r="A6" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>572</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>573</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>574</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="48">
       <c r="A7" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>576</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>577</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>578</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="64">
       <c r="A8" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>579</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>580</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="80">
       <c r="A9" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>581</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>582</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>583</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>584</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="112">
       <c r="A10" s="8" t="s">
+        <v>583</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>584</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>585</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>586</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="96">
       <c r="A11" s="8" t="s">
+        <v>586</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>588</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>589</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>590</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="64">
       <c r="A12" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>590</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>591</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>592</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="64">
       <c r="A13" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>593</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>594</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>595</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="96">
       <c r="A14" s="8" t="s">
+        <v>595</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>597</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>598</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>599</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="80">
       <c r="A15" s="8" t="s">
+        <v>598</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>599</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>600</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>601</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="80">
       <c r="A16" s="8" t="s">
+        <v>601</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>602</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>603</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>604</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>605</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="80">
       <c r="A17" s="8" t="s">
+        <v>604</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>606</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>607</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>608</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="80">
       <c r="A18" s="8" t="s">
+        <v>607</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>608</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>609</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>610</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="112">
       <c r="A19" s="8" t="s">
+        <v>610</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>611</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>612</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>613</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="64">
       <c r="A20" s="8" t="s">
+        <v>613</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>614</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>615</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>616</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>617</v>
       </c>
     </row>
   </sheetData>

</xml_diff>